<commit_message>
Guard Sudoku candidate chain against duplicate forced singles
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{182CCD97-8A25-A94B-BE02-886721ADC980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C047800B-56FC-D04E-9CDA-6D827E4EAB0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3280" yWindow="500" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -87,7 +87,8 @@
     <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,_xlpm.colStep),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,_xlpm.colText),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
     <definedName name="SDKP_ClaimingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.acc,_xlpm.i,IF(_xlpm.acc&lt;&gt;"",_xlpm.acc,_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,0,_xlpm.k),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.rs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.rs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*(_xlpm.band-1),_xlpm.bc,1+3*QUOTIENT(_xlpm.k-1,3),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.cc&lt;&gt;_xlpm.k)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.rs&amp;"C"&amp;_xlpm.k),_xlpm.b,3*(_xlpm.band-1)+1+QUOTIENT(_xlpm.k-1,3),IF(_xlpm.txt&lt;&gt;"","Claiming column · Column "&amp;_xlpm.k&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".","")))))))</definedName>
     <definedName name="SDKP_ClaimingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.acc,_xlpm.i,IF(_xlpm.acc&lt;&gt;"",_xlpm.acc,_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,_xlpm.r,0),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.cs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(,9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.cs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*QUOTIENT(_xlpm.r-1,3),_xlpm.bc,1+3*(_xlpm.band-1),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.rr&lt;&gt;_xlpm.r)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.cs),_xlpm.b,3*QUOTIENT(_xlpm.r-1,3)+_xlpm.band,IF(_xlpm.txt&lt;&gt;"","Claiming row · Row "&amp;_xlpm.r&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".","")))))))</definedName>
-    <definedName name="SDKP_Contradiction">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlfn.LET(_xlpm.conflict,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,--SDK_Conflict(_xlpm.board,_xlpm.r,_xlpm.k))))&gt;0,_xlpm.deadCell,SUM(--((_xlpm.board="")*(_xlpm.c="")))&gt;0,_xlpm.rowMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,_xlpm.r,0)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;"")))=0))))&gt;0,_xlpm.colMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,0,_xlpm.k)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;"")))=0))))&gt;0,_xlpm.boxMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.bv,_xlfn.TOCOL(INDEX(_xlpm.board,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),_xlpm.cv,_xlfn.TOCOL(INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),--AND(SUM(--(_xlpm.bv=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.cv&amp;"")))=0)))))&gt;0,OR(_xlpm.conflict,_xlpm.deadCell,_xlpm.rowMissing,_xlpm.colMissing,_xlpm.boxMissing)))</definedName>
+    <definedName name="SDKP_Contradiction">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlfn.LET(_xlpm.conflict,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,--SDK_Conflict(_xlpm.board,_xlpm.r,_xlpm.k))))&gt;0,_xlpm.deadCell,SUM(--((_xlpm.board="")*(_xlpm.c="")))&gt;0,_xlpm.rowMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,_xlpm.r,0)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;"")))=0))))&gt;0,_xlpm.colMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,0,_xlpm.k)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;"")))=0))))&gt;0,_xlpm.boxMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.bv,_xlfn.TOCOL(INDEX(_xlpm.board,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),_xlpm.cv,_xlfn.TOCOL(INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),--AND(SUM(--(_xlpm.bv=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.cv&amp;"")))=0)))))&gt;0,OR(_xlpm.conflict,_xlpm.deadCell,_xlpm.rowMissing,_xlpm.colMissing,_xlpm.boxMissing,SDKP_ForcedConflict(_xlpm.board,_xlpm.c))))</definedName>
+    <definedName name="SDKP_ForcedConflict">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlfn.LET(_xlpm.forced,IF((_xlpm.board="")*(LEN(_xlpm.c&amp;"")=1),_xlpm.c&amp;"",""),_xlpm.rowBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,--(SUM(--(INDEX(_xlpm.forced,_xlpm.r,0)=_xlpm.d&amp;""))&gt;1))))&gt;0,_xlpm.colBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,--(SUM(--(INDEX(_xlpm.forced,0,_xlpm.k)=_xlpm.d&amp;""))&gt;1))))&gt;0,_xlpm.boxBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.v,_xlfn.TOCOL(INDEX(_xlpm.forced,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),--(SUM(--(_xlpm.v=_xlpm.d&amp;""))&gt;1)))))&gt;0,OR(_xlpm.rowBad,_xlpm.colBad,_xlpm.boxBad)))</definedName>
     <definedName name="SDKP_HiddenBox">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc))&amp;"")))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.b,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.x,_xlfn.TOCOL(INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),_xlpm.q,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.x&amp;""))),_xlpm.r,_xlpm.br+QUOTIENT(_xlpm.q-1,3),_xlpm.k,_xlpm.bc+MOD(_xlpm.q-1,3),"Hidden single in box · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in box "&amp;_xlpm.b&amp;"."))))</definedName>
     <definedName name="SDKP_HiddenCol">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;""))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.r,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;""))),"Hidden single in column · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in column "&amp;_xlpm.k&amp;"."))))</definedName>
     <definedName name="SDKP_HiddenRow">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.k,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))),"Hidden single in row · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in row "&amp;_xlpm.r&amp;"."))))</definedName>
@@ -180,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="903" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="646">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2129,6 +2130,30 @@
   </si>
   <si>
     <t>Pointing-column step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Duplicate forced singles in a row are contradictory</t>
+  </si>
+  <si>
+    <t>Two empty cells in row 1 are both forced to digit 1</t>
+  </si>
+  <si>
+    <t>Duplicate forced singles in a column are contradictory</t>
+  </si>
+  <si>
+    <t>Two empty cells in column 1 are both forced to digit 1</t>
+  </si>
+  <si>
+    <t>Duplicate forced singles in a box are contradictory</t>
+  </si>
+  <si>
+    <t>R1C1 and R2C2 force digit 1 in the same box only</t>
+  </si>
+  <si>
+    <t>Separated forced singles remain viable</t>
+  </si>
+  <si>
+    <t>R1C1 and R4C4 do not share a row, column or box</t>
   </si>
 </sst>
 </file>
@@ -5773,7 +5798,7 @@
       <c r="C45" s="95"/>
       <c r="D45" s="96" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>97 checks passing · 18 on demand</v>
+        <v>101 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="97"/>
       <c r="F45" s="97"/>
@@ -37780,7 +37805,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P168"/>
+  <dimension ref="A1:P172"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -40850,6 +40875,82 @@
       </c>
       <c r="E168" t="str">
         <f>IF(D168=C168,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5">
+      <c r="A169" t="s">
+        <v>638</v>
+      </c>
+      <c r="B169" t="s">
+        <v>639</v>
+      </c>
+      <c r="C169" t="b">
+        <v>1</v>
+      </c>
+      <c r="D169" t="b" cm="1">
+        <f t="array" ref="D169">_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.cand,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,OR(_xlpm.k=1,_xlpm.k=2)),"1","123456789"))),SDKP_Contradiction(_xlpm.board,_xlpm.cand))</f>
+        <v>1</v>
+      </c>
+      <c r="E169" t="str">
+        <f>IF(D169=C169,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5">
+      <c r="A170" t="s">
+        <v>640</v>
+      </c>
+      <c r="B170" t="s">
+        <v>641</v>
+      </c>
+      <c r="C170" t="b">
+        <v>1</v>
+      </c>
+      <c r="D170" t="b" cm="1">
+        <f t="array" ref="D170">_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.cand,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.k=1,OR(_xlpm.r=1,_xlpm.r=2)),"1","123456789"))),SDKP_Contradiction(_xlpm.board,_xlpm.cand))</f>
+        <v>1</v>
+      </c>
+      <c r="E170" t="str">
+        <f>IF(D170=C170,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5">
+      <c r="A171" t="s">
+        <v>642</v>
+      </c>
+      <c r="B171" t="s">
+        <v>643</v>
+      </c>
+      <c r="C171" t="b">
+        <v>1</v>
+      </c>
+      <c r="D171" t="b" cm="1">
+        <f t="array" ref="D171">_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.cand,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(OR(AND(_xlpm.r=1,_xlpm.k=1),AND(_xlpm.r=2,_xlpm.k=2)),"1","123456789"))),SDKP_Contradiction(_xlpm.board,_xlpm.cand))</f>
+        <v>1</v>
+      </c>
+      <c r="E171" t="str">
+        <f>IF(D171=C171,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5">
+      <c r="A172" t="s">
+        <v>644</v>
+      </c>
+      <c r="B172" t="s">
+        <v>645</v>
+      </c>
+      <c r="C172" t="b">
+        <v>0</v>
+      </c>
+      <c r="D172" t="b" cm="1">
+        <f t="array" ref="D172">_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.cand,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(OR(AND(_xlpm.r=1,_xlpm.k=1),AND(_xlpm.r=4,_xlpm.k=4)),"1","123456789"))),SDKP_Contradiction(_xlpm.board,_xlpm.cand))</f>
+        <v>0</v>
+      </c>
+      <c r="E172" t="str">
+        <f>IF(D172=C172,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Stop Sudoku candidate chain when elimination makes no progress
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C047800B-56FC-D04E-9CDA-6D827E4EAB0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0592BFA9-81FA-E742-A64D-7E5251C79B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3280" yWindow="500" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -84,11 +84,12 @@
     <definedName name="SDKP_ApplyStep">_xlfn.LAMBDA(_xlpm.c,_xlpm.s,_xlfn.LET(_xlpm.removeText,INDEX(_xlpm.s,1,3)&amp;"",_xlpm.targets,INDEX(_xlpm.s,1,4)&amp;"",_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.LET(_xlpm.cur,INDEX(_xlpm.c,_xlpm.r,_xlpm.k)&amp;"",_xlpm.coord,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k,IF(OR(_xlpm.cur="",ISERROR(SEARCH(_xlpm.coord,_xlpm.targets))),_xlpm.cur,_xlfn.LET(_xlpm.chars,MID(_xlpm.cur,_xlfn.SEQUENCE(LEN(_xlpm.cur)),1),_xlfn.TEXTJOIN("",TRUE,_xlfn._xlws.FILTER(_xlpm.chars,ISERROR(SEARCH(_xlpm.chars,_xlpm.removeText)),"")))))))))</definedName>
     <definedName name="SDKP_BasicHint">_xlfn.LAMBDA(_xlpm.c,_xlfn.LET(_xlpm.a,SDKP_Naked(_xlpm.c),_xlpm.b,SDKP_HiddenRow(_xlpm.c),_xlpm.d,SDKP_HiddenCol(_xlpm.c),_xlpm.e,SDKP_HiddenBox(_xlpm.c),IF(_xlpm.a&lt;&gt;"",_xlpm.a,IF(_xlpm.b&lt;&gt;"",_xlpm.b,IF(_xlpm.d&lt;&gt;"",_xlpm.d,_xlpm.e)))))</definedName>
     <definedName name="SDKP_Chain">_xlfn.LAMBDA(_xlpm.board,_xlpm.lim,SDKP_ChainLoop(_xlpm.board,SDK_CandidateMatrix(_xlpm.board),0,_xlpm.lim,""))</definedName>
-    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,_xlpm.colStep),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,_xlpm.colText),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
+    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,_xlpm.colStep),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,_xlpm.colText),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
     <definedName name="SDKP_ClaimingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.acc,_xlpm.i,IF(_xlpm.acc&lt;&gt;"",_xlpm.acc,_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,0,_xlpm.k),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.rs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.rs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*(_xlpm.band-1),_xlpm.bc,1+3*QUOTIENT(_xlpm.k-1,3),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.cc&lt;&gt;_xlpm.k)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.rs&amp;"C"&amp;_xlpm.k),_xlpm.b,3*(_xlpm.band-1)+1+QUOTIENT(_xlpm.k-1,3),IF(_xlpm.txt&lt;&gt;"","Claiming column · Column "&amp;_xlpm.k&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".","")))))))</definedName>
     <definedName name="SDKP_ClaimingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.acc,_xlpm.i,IF(_xlpm.acc&lt;&gt;"",_xlpm.acc,_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,_xlpm.r,0),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.cs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(,9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.cs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*QUOTIENT(_xlpm.r-1,3),_xlpm.bc,1+3*(_xlpm.band-1),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.rr&lt;&gt;_xlpm.r)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.cs),_xlpm.b,3*QUOTIENT(_xlpm.r-1,3)+_xlpm.band,IF(_xlpm.txt&lt;&gt;"","Claiming row · Row "&amp;_xlpm.r&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".","")))))))</definedName>
     <definedName name="SDKP_Contradiction">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlfn.LET(_xlpm.conflict,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,--SDK_Conflict(_xlpm.board,_xlpm.r,_xlpm.k))))&gt;0,_xlpm.deadCell,SUM(--((_xlpm.board="")*(_xlpm.c="")))&gt;0,_xlpm.rowMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,_xlpm.r,0)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;"")))=0))))&gt;0,_xlpm.colMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,0,_xlpm.k)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;"")))=0))))&gt;0,_xlpm.boxMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.bv,_xlfn.TOCOL(INDEX(_xlpm.board,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),_xlpm.cv,_xlfn.TOCOL(INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),--AND(SUM(--(_xlpm.bv=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.cv&amp;"")))=0)))))&gt;0,OR(_xlpm.conflict,_xlpm.deadCell,_xlpm.rowMissing,_xlpm.colMissing,_xlpm.boxMissing,SDKP_ForcedConflict(_xlpm.board,_xlpm.c))))</definedName>
     <definedName name="SDKP_ForcedConflict">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlfn.LET(_xlpm.forced,IF((_xlpm.board="")*(LEN(_xlpm.c&amp;"")=1),_xlpm.c&amp;"",""),_xlpm.rowBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,--(SUM(--(INDEX(_xlpm.forced,_xlpm.r,0)=_xlpm.d&amp;""))&gt;1))))&gt;0,_xlpm.colBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,--(SUM(--(INDEX(_xlpm.forced,0,_xlpm.k)=_xlpm.d&amp;""))&gt;1))))&gt;0,_xlpm.boxBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.v,_xlfn.TOCOL(INDEX(_xlpm.forced,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),--(SUM(--(_xlpm.v=_xlpm.d&amp;""))&gt;1)))))&gt;0,OR(_xlpm.rowBad,_xlpm.colBad,_xlpm.boxBad)))</definedName>
+    <definedName name="SDKP_HasProgress">_xlfn.LAMBDA(_xlpm.before,_xlpm.after,SUM(LEN(_xlpm.after&amp;""))&lt;SUM(LEN(_xlpm.before&amp;"")))</definedName>
     <definedName name="SDKP_HiddenBox">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc))&amp;"")))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.b,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.x,_xlfn.TOCOL(INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),_xlpm.q,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.x&amp;""))),_xlpm.r,_xlpm.br+QUOTIENT(_xlpm.q-1,3),_xlpm.k,_xlpm.bc+MOD(_xlpm.q-1,3),"Hidden single in box · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in box "&amp;_xlpm.b&amp;"."))))</definedName>
     <definedName name="SDKP_HiddenCol">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;""))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.r,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;""))),"Hidden single in column · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in column "&amp;_xlpm.k&amp;"."))))</definedName>
     <definedName name="SDKP_HiddenRow">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.k,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))),"Hidden single in row · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in row "&amp;_xlpm.r&amp;"."))))</definedName>
@@ -181,7 +182,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="646">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="652">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2154,6 +2155,24 @@
   </si>
   <si>
     <t>R1C1 and R4C4 do not share a row, column or box</t>
+  </si>
+  <si>
+    <t>No-op elimination must not count as chain progress</t>
+  </si>
+  <si>
+    <t>Removing absent digit 9 leaves R1C1 candidates 12</t>
+  </si>
+  <si>
+    <t>Effective elimination counts as chain progress</t>
+  </si>
+  <si>
+    <t>Removing digit 1 changes R1C1 candidates 12 to 2</t>
+  </si>
+  <si>
+    <t>Candidate expansion must not count as progress</t>
+  </si>
+  <si>
+    <t>Growing R1C1 from 12 to 123 cannot continue the chain</t>
   </si>
 </sst>
 </file>
@@ -5798,7 +5817,7 @@
       <c r="C45" s="95"/>
       <c r="D45" s="96" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>101 checks passing · 18 on demand</v>
+        <v>104 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="97"/>
       <c r="F45" s="97"/>
@@ -37805,7 +37824,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P172"/>
+  <dimension ref="A1:P175"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -40951,6 +40970,63 @@
       </c>
       <c r="E172" t="str">
         <f>IF(D172=C172,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5">
+      <c r="A173" t="s">
+        <v>646</v>
+      </c>
+      <c r="B173" t="s">
+        <v>647</v>
+      </c>
+      <c r="C173" t="b">
+        <v>1</v>
+      </c>
+      <c r="D173" t="b" cm="1">
+        <f t="array" ref="D173">_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"12",""))),_xlpm.s,_xlfn.HSTACK("Pointing row","R1C2","9","R1C1","probe"),_xlpm.next,SDKP_ApplyStep(_xlpm.c,_xlpm.s),IFERROR(AND(INDEX(_xlpm.next,1,1)="12",NOT(SDKP_HasProgress(_xlpm.c,_xlpm.next))),FALSE))</f>
+        <v>1</v>
+      </c>
+      <c r="E173" t="str">
+        <f>IF(D173=C173,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5">
+      <c r="A174" t="s">
+        <v>648</v>
+      </c>
+      <c r="B174" t="s">
+        <v>649</v>
+      </c>
+      <c r="C174" t="b">
+        <v>1</v>
+      </c>
+      <c r="D174" t="b" cm="1">
+        <f t="array" ref="D174">_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"12",""))),_xlpm.s,_xlfn.HSTACK("Pointing row","R1C2","1","R1C1","probe"),_xlpm.next,SDKP_ApplyStep(_xlpm.c,_xlpm.s),IFERROR(AND(INDEX(_xlpm.next,1,1)="2",SDKP_HasProgress(_xlpm.c,_xlpm.next)),FALSE))</f>
+        <v>1</v>
+      </c>
+      <c r="E174" t="str">
+        <f>IF(D174=C174,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5">
+      <c r="A175" t="s">
+        <v>650</v>
+      </c>
+      <c r="B175" t="s">
+        <v>651</v>
+      </c>
+      <c r="C175" t="b">
+        <v>1</v>
+      </c>
+      <c r="D175" t="b" cm="1">
+        <f t="array" ref="D175">_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"12",""))),_xlpm.next,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"123",""))),IFERROR(NOT(SDKP_HasProgress(_xlpm.c,_xlpm.next)),FALSE))</f>
+        <v>1</v>
+      </c>
+      <c r="E175" t="str">
+        <f>IF(D175=C175,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate Sudoku prototype Claiming Row to structured step
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0592BFA9-81FA-E742-A64D-7E5251C79B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F303E99-F656-4C41-8793-3429C93D123E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3280" yWindow="500" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -84,9 +84,10 @@
     <definedName name="SDKP_ApplyStep">_xlfn.LAMBDA(_xlpm.c,_xlpm.s,_xlfn.LET(_xlpm.removeText,INDEX(_xlpm.s,1,3)&amp;"",_xlpm.targets,INDEX(_xlpm.s,1,4)&amp;"",_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.LET(_xlpm.cur,INDEX(_xlpm.c,_xlpm.r,_xlpm.k)&amp;"",_xlpm.coord,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k,IF(OR(_xlpm.cur="",ISERROR(SEARCH(_xlpm.coord,_xlpm.targets))),_xlpm.cur,_xlfn.LET(_xlpm.chars,MID(_xlpm.cur,_xlfn.SEQUENCE(LEN(_xlpm.cur)),1),_xlfn.TEXTJOIN("",TRUE,_xlfn._xlws.FILTER(_xlpm.chars,ISERROR(SEARCH(_xlpm.chars,_xlpm.removeText)),"")))))))))</definedName>
     <definedName name="SDKP_BasicHint">_xlfn.LAMBDA(_xlpm.c,_xlfn.LET(_xlpm.a,SDKP_Naked(_xlpm.c),_xlpm.b,SDKP_HiddenRow(_xlpm.c),_xlpm.d,SDKP_HiddenCol(_xlpm.c),_xlpm.e,SDKP_HiddenBox(_xlpm.c),IF(_xlpm.a&lt;&gt;"",_xlpm.a,IF(_xlpm.b&lt;&gt;"",_xlpm.b,IF(_xlpm.d&lt;&gt;"",_xlpm.d,_xlpm.e)))))</definedName>
     <definedName name="SDKP_Chain">_xlfn.LAMBDA(_xlpm.board,_xlpm.lim,SDKP_ChainLoop(_xlpm.board,SDK_CandidateMatrix(_xlpm.board),0,_xlpm.lim,""))</definedName>
-    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,_xlpm.colStep),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,_xlpm.colText),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
+    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.claimRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingRowStep(_xlpm.c)),_xlpm.claimRowText,INDEX(_xlpm.claimRowStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,IF(_xlpm.colText&lt;&gt;"",_xlpm.colStep,_xlpm.claimRowStep)),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,IF(_xlpm.colText&lt;&gt;"",_xlpm.colText,_xlpm.claimRowText)),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
     <definedName name="SDKP_ClaimingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.acc,_xlpm.i,IF(_xlpm.acc&lt;&gt;"",_xlpm.acc,_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,0,_xlpm.k),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.rs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.rs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*(_xlpm.band-1),_xlpm.bc,1+3*QUOTIENT(_xlpm.k-1,3),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.cc&lt;&gt;_xlpm.k)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.rs&amp;"C"&amp;_xlpm.k),_xlpm.b,3*(_xlpm.band-1)+1+QUOTIENT(_xlpm.k-1,3),IF(_xlpm.txt&lt;&gt;"","Claiming column · Column "&amp;_xlpm.k&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".","")))))))</definedName>
-    <definedName name="SDKP_ClaimingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.acc,_xlpm.i,IF(_xlpm.acc&lt;&gt;"",_xlpm.acc,_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,_xlpm.r,0),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.cs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(,9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.cs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*QUOTIENT(_xlpm.r-1,3),_xlpm.bc,1+3*(_xlpm.band-1),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.rr&lt;&gt;_xlpm.r)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.cs),_xlpm.b,3*QUOTIENT(_xlpm.r-1,3)+_xlpm.band,IF(_xlpm.txt&lt;&gt;"","Claiming row · Row "&amp;_xlpm.r&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".","")))))))</definedName>
+    <definedName name="SDKP_ClaimingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_ClaimingRowStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_ClaimingRowStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.i,_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,_xlpm.r,0),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.cs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(,9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.cs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*QUOTIENT(_xlpm.r-1,3),_xlpm.bc,1+3*(_xlpm.band-1),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.rr&lt;&gt;_xlpm.r)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.cs),_xlpm.b,3*QUOTIENT(_xlpm.r-1,3)+_xlpm.band,_xlpm.displayText,"Claiming row · Row "&amp;_xlpm.r&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".",IF(_xlpm.txt&lt;&gt;"",_xlfn.HSTACK("Claiming row",_xlpm.sourceText,_xlpm.d&amp;"",_xlpm.txt,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_Contradiction">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlfn.LET(_xlpm.conflict,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,--SDK_Conflict(_xlpm.board,_xlpm.r,_xlpm.k))))&gt;0,_xlpm.deadCell,SUM(--((_xlpm.board="")*(_xlpm.c="")))&gt;0,_xlpm.rowMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,_xlpm.r,0)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;"")))=0))))&gt;0,_xlpm.colMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,0,_xlpm.k)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;"")))=0))))&gt;0,_xlpm.boxMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.bv,_xlfn.TOCOL(INDEX(_xlpm.board,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),_xlpm.cv,_xlfn.TOCOL(INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),--AND(SUM(--(_xlpm.bv=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.cv&amp;"")))=0)))))&gt;0,OR(_xlpm.conflict,_xlpm.deadCell,_xlpm.rowMissing,_xlpm.colMissing,_xlpm.boxMissing,SDKP_ForcedConflict(_xlpm.board,_xlpm.c))))</definedName>
     <definedName name="SDKP_ForcedConflict">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlfn.LET(_xlpm.forced,IF((_xlpm.board="")*(LEN(_xlpm.c&amp;"")=1),_xlpm.c&amp;"",""),_xlpm.rowBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,--(SUM(--(INDEX(_xlpm.forced,_xlpm.r,0)=_xlpm.d&amp;""))&gt;1))))&gt;0,_xlpm.colBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,--(SUM(--(INDEX(_xlpm.forced,0,_xlpm.k)=_xlpm.d&amp;""))&gt;1))))&gt;0,_xlpm.boxBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.v,_xlfn.TOCOL(INDEX(_xlpm.forced,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),--(SUM(--(_xlpm.v=_xlpm.d&amp;""))&gt;1)))))&gt;0,OR(_xlpm.rowBad,_xlpm.colBad,_xlpm.boxBad)))</definedName>
     <definedName name="SDKP_HasProgress">_xlfn.LAMBDA(_xlpm.before,_xlpm.after,SUM(LEN(_xlpm.after&amp;""))&lt;SUM(LEN(_xlpm.before&amp;"")))</definedName>
@@ -182,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="652">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="657">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2173,6 +2174,21 @@
   </si>
   <si>
     <t>Growing R1C1 from 12 to 123 cannot continue the chain</t>
+  </si>
+  <si>
+    <t>Claiming-row step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Structured Claiming-row apply ignores display wording</t>
+  </si>
+  <si>
+    <t>Digit and target fields, not prose, remove 3 from R3C7</t>
+  </si>
+  <si>
+    <t>Claiming-row public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Public wrapper returns structured field 5</t>
   </si>
 </sst>
 </file>
@@ -5817,7 +5833,7 @@
       <c r="C45" s="95"/>
       <c r="D45" s="96" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>104 checks passing · 18 on demand</v>
+        <v>107 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="97"/>
       <c r="F45" s="97"/>
@@ -37824,7 +37840,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P175"/>
+  <dimension ref="A1:P178"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -41027,6 +41043,63 @@
       </c>
       <c r="E175" t="str">
         <f>IF(D175=C175,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5">
+      <c r="A176" t="s">
+        <v>652</v>
+      </c>
+      <c r="B176" t="s">
+        <v>630</v>
+      </c>
+      <c r="C176" t="b">
+        <v>1</v>
+      </c>
+      <c r="D176" t="b" cm="1">
+        <f t="array" ref="D176">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=2,OR(_xlpm.k=7,_xlpm.k=8)),"13",AND(_xlpm.r=3,_xlpm.k=7),"34",AND(_xlpm.r=2,_xlpm.k&lt;&gt;7,_xlpm.k&lt;&gt;8),"12456789",AND(OR(_xlpm.r=1,_xlpm.r=3),_xlpm.k&gt;=7,_xlpm.k&lt;=9),"12456789",TRUE,"123456789"))),_xlpm.s,SDKP_ClaimingRowStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Claiming row",INDEX(_xlpm.s,1,2)="R2C7, R2C8",INDEX(_xlpm.s,1,3)="3",INDEX(_xlpm.s,1,4)="R3C7",INDEX(_xlpm.s,1,5)="Claiming row · Row 2 confines digit 3 to box 3 via R2C7, R2C8 · Remove 3 from R3C7."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E176" t="str">
+        <f>IF(D176=C176,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5">
+      <c r="A177" t="s">
+        <v>653</v>
+      </c>
+      <c r="B177" t="s">
+        <v>654</v>
+      </c>
+      <c r="C177" t="b">
+        <v>1</v>
+      </c>
+      <c r="D177" t="b" cm="1">
+        <f t="array" ref="D177">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=2,OR(_xlpm.k=7,_xlpm.k=8)),"13",AND(_xlpm.r=3,_xlpm.k=7),"34",AND(_xlpm.r=2,_xlpm.k&lt;&gt;7,_xlpm.k&lt;&gt;8),"12456789",AND(OR(_xlpm.r=1,_xlpm.r=3),_xlpm.k&gt;=7,_xlpm.k&lt;=9),"12456789",TRUE,"123456789"))),_xlpm.s,SDKP_ClaimingRowStep(_xlpm.c),_xlpm.t,_xlfn.HSTACK(INDEX(_xlpm.s,1,1),INDEX(_xlpm.s,1,2),INDEX(_xlpm.s,1,3),INDEX(_xlpm.s,1,4),"wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.c,_xlpm.t),AND(INDEX(_xlpm.after,3,7)="4",INDEX(_xlpm.after,2,7)="13")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E177" t="str">
+        <f>IF(D177=C177,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5">
+      <c r="A178" t="s">
+        <v>655</v>
+      </c>
+      <c r="B178" t="s">
+        <v>656</v>
+      </c>
+      <c r="C178" t="b">
+        <v>1</v>
+      </c>
+      <c r="D178" t="b" cm="1">
+        <f t="array" ref="D178">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=2,OR(_xlpm.k=7,_xlpm.k=8)),"13",AND(_xlpm.r=3,_xlpm.k=7),"34",AND(_xlpm.r=2,_xlpm.k&lt;&gt;7,_xlpm.k&lt;&gt;8),"12456789",AND(OR(_xlpm.r=1,_xlpm.r=3),_xlpm.k&gt;=7,_xlpm.k&lt;=9),"12456789",TRUE,"123456789"))),_xlpm.s,SDKP_ClaimingRowStep(_xlpm.c),SDKP_ClaimingRow(_xlpm.c)=INDEX(_xlpm.s,1,5)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E178" t="str">
+        <f>IF(D178=C178,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate Sudoku prototype Naked Pair Row to structured step
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D61D5FA-C796-7C4F-B2D9-3CB4891736C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{872FFCB4-8498-1641-A2F4-481DDC0891D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -84,7 +84,7 @@
     <definedName name="SDKP_ApplyStep">_xlfn.LAMBDA(_xlpm.c,_xlpm.s,_xlfn.LET(_xlpm.removeText,INDEX(_xlpm.s,1,3)&amp;"",_xlpm.targets,INDEX(_xlpm.s,1,4)&amp;"",_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.LET(_xlpm.cur,INDEX(_xlpm.c,_xlpm.r,_xlpm.k)&amp;"",_xlpm.coord,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k,IF(OR(_xlpm.cur="",ISERROR(SEARCH(_xlpm.coord,_xlpm.targets))),_xlpm.cur,_xlfn.LET(_xlpm.chars,MID(_xlpm.cur,_xlfn.SEQUENCE(LEN(_xlpm.cur)),1),_xlfn.TEXTJOIN("",TRUE,_xlfn._xlws.FILTER(_xlpm.chars,ISERROR(SEARCH(_xlpm.chars,_xlpm.removeText)),"")))))))))</definedName>
     <definedName name="SDKP_BasicHint">_xlfn.LAMBDA(_xlpm.c,_xlfn.LET(_xlpm.a,SDKP_Naked(_xlpm.c),_xlpm.b,SDKP_HiddenRow(_xlpm.c),_xlpm.d,SDKP_HiddenCol(_xlpm.c),_xlpm.e,SDKP_HiddenBox(_xlpm.c),IF(_xlpm.a&lt;&gt;"",_xlpm.a,IF(_xlpm.b&lt;&gt;"",_xlpm.b,IF(_xlpm.d&lt;&gt;"",_xlpm.d,_xlpm.e)))))</definedName>
     <definedName name="SDKP_Chain">_xlfn.LAMBDA(_xlpm.board,_xlpm.lim,SDKP_ChainLoop(_xlpm.board,SDK_CandidateMatrix(_xlpm.board),0,_xlpm.lim,""))</definedName>
-    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.claimRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingRowStep(_xlpm.c)),_xlpm.claimRowText,INDEX(_xlpm.claimRowStep,1,5),_xlpm.claimColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingColStep(_xlpm.c)),_xlpm.claimColText,INDEX(_xlpm.claimColStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,IF(_xlpm.colText&lt;&gt;"",_xlpm.colStep,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowStep,_xlpm.claimColStep))),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,IF(_xlpm.colText&lt;&gt;"",_xlpm.colText,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowText,_xlpm.claimColText))),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
+    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.claimRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingRowStep(_xlpm.c)),_xlpm.claimRowText,INDEX(_xlpm.claimRowStep,1,5),_xlpm.claimColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingColStep(_xlpm.c)),_xlpm.claimColText,INDEX(_xlpm.claimColStep,1,5),_xlpm.pairRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairRowStep(_xlpm.c)),_xlpm.pairRowText,INDEX(_xlpm.pairRowStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,IF(_xlpm.colText&lt;&gt;"",_xlpm.colStep,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowStep,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColStep,_xlpm.pairRowStep)))),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,IF(_xlpm.colText&lt;&gt;"",_xlpm.colText,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowText,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColText,_xlpm.pairRowText)))),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
     <definedName name="SDKP_ClaimingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_ClaimingColStep(_xlpm.inputCandidates),1,5))</definedName>
     <definedName name="SDKP_ClaimingColStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.i,_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,0,_xlpm.k),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.rs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.rs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*(_xlpm.band-1),_xlpm.bc,1+3*QUOTIENT(_xlpm.k-1,3),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.cc&lt;&gt;_xlpm.k)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.rs&amp;"C"&amp;_xlpm.k),_xlpm.b,3*(_xlpm.band-1)+1+QUOTIENT(_xlpm.k-1,3),_xlpm.displayText,"Claiming column · Column "&amp;_xlpm.k&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".",IF(_xlpm.txt&lt;&gt;"",_xlfn.HSTACK("Claiming column",_xlpm.sourceText,_xlpm.d&amp;"",_xlpm.txt,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_ClaimingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_ClaimingRowStep(_xlpm.inputCandidates),1,5))</definedName>
@@ -98,7 +98,8 @@
     <definedName name="SDKP_Naked">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.m,LEN(_xlpm.c)=1,_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlfn.TOCOL(_xlpm.m)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.k,MOD(_xlpm.p-1,9)+1,_xlpm.d,INDEX(_xlpm.c,_xlpm.r,_xlpm.k),"Naked single · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · This is the only legal candidate remaining in the square."))))</definedName>
     <definedName name="SDKP_NakedPairBox">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.foundHint,_xlpm.scanIndex,IF(_xlpm.foundHint&lt;&gt;"",_xlpm.foundHint,_xlfn.LET(_xlpm.rowNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.colNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.boxStartRow,1+3*QUOTIENT(_xlpm.rowNum-1,3),_xlpm.boxStartCol,1+3*QUOTIENT(_xlpm.colNum-1,3),_xlpm.unitVals,_xlfn.TOCOL(INDEX(_xlpm.candMatrix,_xlfn.SEQUENCE(3,,_xlpm.boxStartRow),_xlfn.SEQUENCE(,3,_xlpm.boxStartCol)))&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.rowCoords,_xlpm.boxStartRow+QUOTIENT(_xlfn.SEQUENCE(9)-1,3),_xlpm.colCoords,_xlpm.boxStartCol+MOD(_xlfn.SEQUENCE(9)-1,3),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstIndex)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondIndex),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowCoords&amp;"C"&amp;_xlpm.colCoords,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.firstRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.firstIndex-1,3),_xlpm.firstCol,_xlpm.boxStartCol+MOD(_xlpm.firstIndex-1,3),_xlpm.secondRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.secondIndex-1,3),_xlpm.secondCol,_xlpm.boxStartCol+MOD(_xlpm.secondIndex-1,3),_xlpm.boxNum,1+3*QUOTIENT(_xlpm.rowNum-1,3)+QUOTIENT(_xlpm.colNum-1,3),IF(_xlpm.targetText&lt;&gt;"","Naked pair in box · R"&amp;_xlpm.firstRow&amp;"C"&amp;_xlpm.firstCol&amp;" and R"&amp;_xlpm.secondRow&amp;"C"&amp;_xlpm.secondCol&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" in box "&amp;_xlpm.boxNum&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".","")))))))</definedName>
     <definedName name="SDKP_NakedPairCol">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.foundHint,_xlpm.scanIndex,IF(_xlpm.foundHint&lt;&gt;"",_xlpm.foundHint,_xlfn.LET(_xlpm.colNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.rowNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.unitVals,INDEX(_xlpm.candMatrix,0,_xlpm.colNum)&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstPos)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondPos),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlfn.SEQUENCE(9)&amp;"C"&amp;_xlpm.colNum,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),IF(_xlpm.targetText&lt;&gt;"","Naked pair in column · R"&amp;_xlpm.firstPos&amp;"C"&amp;_xlpm.colNum&amp;" and R"&amp;_xlpm.secondPos&amp;"C"&amp;_xlpm.colNum&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".","")))))))</definedName>
-    <definedName name="SDKP_NakedPairRow">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.foundHint,_xlpm.scanIndex,IF(_xlpm.foundHint&lt;&gt;"",_xlpm.foundHint,_xlfn.LET(_xlpm.rowNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.colNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.unitVals,INDEX(_xlpm.candMatrix,_xlpm.rowNum,0)&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(,9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1,1),0),_xlpm.secondPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1,COLUMNS(_xlpm.pairPositions)),0),_xlpm.otherMask,(_xlfn.SEQUENCE(,9)&lt;&gt;_xlpm.firstPos)*(_xlfn.SEQUENCE(,9)&lt;&gt;_xlpm.secondPos),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(,9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlfn.SEQUENCE(,9),_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),IF(_xlpm.targetText&lt;&gt;"","Naked pair in row · R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.firstPos&amp;" and R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.secondPos&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".","")))))))</definedName>
+    <definedName name="SDKP_NakedPairRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_NakedPairRowStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_NakedPairRowStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.rowNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.colNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.unitVals,INDEX(_xlpm.candMatrix,_xlpm.rowNum,0)&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(,9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1,1),0),_xlpm.secondPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1,COLUMNS(_xlpm.pairPositions)),0),_xlpm.otherMask,(_xlfn.SEQUENCE(,9)&lt;&gt;_xlpm.firstPos)*(_xlfn.SEQUENCE(,9)&lt;&gt;_xlpm.secondPos),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(,9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlfn.SEQUENCE(,9),_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.sourceText,"R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.firstPos&amp;", R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.secondPos,_xlpm.displayText,"Naked pair in row · R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.firstPos&amp;" and R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.secondPos&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".",IF(_xlpm.targetText&lt;&gt;"",_xlfn.HSTACK("Naked pair in row",_xlpm.sourceText,_xlpm.pairText,_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_PointingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_PointingColStep(_xlpm.inputCandidates),1,5))</definedName>
     <definedName name="SDKP_PointingColStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.boxNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.digitNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.boxStartRow,1+3*QUOTIENT(_xlpm.boxNum-1,3),_xlpm.boxStartCol,1+3*MOD(_xlpm.boxNum-1,3),_xlpm.boxCandidates,INDEX(_xlpm.candMatrix,_xlfn.SEQUENCE(3,,_xlpm.boxStartRow),_xlfn.SEQUENCE(,3,_xlpm.boxStartCol)),_xlpm.candidateMask,ISNUMBER(SEARCH(_xlpm.digitNum&amp;"",_xlpm.boxCandidates&amp;"")),_xlpm.candidateCount,SUM(--_xlpm.candidateMask),_xlpm.rowCoordinates,_xlfn.TOCOL(_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.rowOffset,_xlpm.colOffset,_xlpm.boxStartRow+_xlpm.rowOffset-1))),_xlpm.colCoordinates,_xlfn.TOCOL(_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.rowOffset,_xlpm.colOffset,_xlpm.boxStartCol+_xlpm.colOffset-1))),_xlpm.candidateCols,_xlfn._xlws.FILTER(_xlpm.colCoordinates,_xlfn.TOCOL(_xlpm.candidateMask),""),_xlpm.sourceCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowCoordinates&amp;"C"&amp;_xlpm.colCoordinates,_xlfn.TOCOL(_xlpm.candidateMask),""),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.sourceCells),_xlpm.singleCol,IF(_xlpm.candidateCount&gt;1,MIN(_xlpm.candidateCols)=MAX(_xlpm.candidateCols),FALSE),_xlpm.targetCol,IF(_xlpm.singleCol,INDEX(_xlpm.candidateCols,1),1),_xlpm.colCandidates,_xlfn.CHOOSECOLS(_xlpm.candMatrix,_xlpm.targetCol)&amp;"",_xlpm.rowNumbers,_xlfn.SEQUENCE(9),_xlpm.outsideMask,((_xlpm.rowNumbers&lt;_xlpm.boxStartRow)+(_xlpm.rowNumbers&gt;_xlpm.boxStartRow+2))&gt;0,_xlpm.containsMask,ISNUMBER(SEARCH(_xlpm.digitNum&amp;"",_xlpm.colCandidates)),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowNumbers&amp;"C"&amp;_xlpm.targetCol,_xlpm.outsideMask*_xlpm.containsMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.displayText,"Pointing column · Box "&amp;_xlpm.boxNum&amp;" confines digit "&amp;_xlpm.digitNum&amp;" to column "&amp;_xlpm.targetCol&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.digitNum&amp;" from "&amp;_xlpm.targetText&amp;".",IF(AND(_xlpm.singleCol,_xlpm.targetText&lt;&gt;""),_xlfn.HSTACK("Pointing column",_xlpm.sourceText,_xlpm.digitNum&amp;"",_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_PointingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_PointingRowStep(_xlpm.inputCandidates),1,5))</definedName>
@@ -184,7 +185,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="929" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="669">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2202,6 +2203,30 @@
   </si>
   <si>
     <t>Claiming-column public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Naked-pair-row step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Pair sources, digits, target and display text stay separate</t>
+  </si>
+  <si>
+    <t>Structured naked-pair-row apply ignores wording</t>
+  </si>
+  <si>
+    <t>Pair digits and target remove 4/7 from R4C7</t>
+  </si>
+  <si>
+    <t>Naked-pair-row public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Old entry returns structured display field</t>
+  </si>
+  <si>
+    <t>Three matching pairs do not form a naked pair</t>
+  </si>
+  <si>
+    <t>Exactly two matching cells are required</t>
   </si>
 </sst>
 </file>
@@ -5846,7 +5871,7 @@
       <c r="C45" s="81"/>
       <c r="D45" s="77" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>110 checks passing · 18 on demand</v>
+        <v>114 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="78"/>
       <c r="F45" s="78"/>
@@ -37853,7 +37878,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P181"/>
+  <dimension ref="A1:P185"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -41170,6 +41195,82 @@
       </c>
       <c r="E181" t="str">
         <f>IF(D181=C181,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5">
+      <c r="A182" t="s">
+        <v>661</v>
+      </c>
+      <c r="B182" t="s">
+        <v>662</v>
+      </c>
+      <c r="C182" t="b">
+        <v>1</v>
+      </c>
+      <c r="D182" t="b" cm="1">
+        <f t="array" ref="D182">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,OR(_xlpm.k=2,_xlpm.k=5)),"47",AND(_xlpm.r=4,_xlpm.k=7),"478",_xlpm.r=4,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairRowStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Naked pair in row",INDEX(_xlpm.s,1,2)="R4C2, R4C5",INDEX(_xlpm.s,1,3)="47",INDEX(_xlpm.s,1,4)="R4C7",INDEX(_xlpm.s,1,5)="Naked pair in row · R4C2 and R4C5 contain only 4/7 · Remove 4 and 7 from R4C7."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E182" t="str">
+        <f>IF(D182=C182,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5">
+      <c r="A183" t="s">
+        <v>663</v>
+      </c>
+      <c r="B183" t="s">
+        <v>664</v>
+      </c>
+      <c r="C183" t="b">
+        <v>1</v>
+      </c>
+      <c r="D183" t="b" cm="1">
+        <f t="array" ref="D183">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,OR(_xlpm.k=2,_xlpm.k=5)),"47",AND(_xlpm.r=4,_xlpm.k=7),"478",_xlpm.r=4,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairRowStep(_xlpm.c),_xlpm.t,_xlfn.HSTACK(INDEX(_xlpm.s,1,1),INDEX(_xlpm.s,1,2),INDEX(_xlpm.s,1,3),INDEX(_xlpm.s,1,4),"wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.c,_xlpm.t),AND(INDEX(_xlpm.after,4,7)="8",INDEX(_xlpm.after,4,2)="47")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E183" t="str">
+        <f>IF(D183=C183,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5">
+      <c r="A184" t="s">
+        <v>665</v>
+      </c>
+      <c r="B184" t="s">
+        <v>666</v>
+      </c>
+      <c r="C184" t="b">
+        <v>1</v>
+      </c>
+      <c r="D184" t="b" cm="1">
+        <f t="array" ref="D184">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,OR(_xlpm.k=2,_xlpm.k=5)),"47",AND(_xlpm.r=4,_xlpm.k=7),"478",_xlpm.r=4,"1235689",TRUE,"123456789"))),SDKP_NakedPairRow(_xlpm.c)=INDEX(SDKP_NakedPairRowStep(_xlpm.c),1,5)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E184" t="str">
+        <f>IF(D184=C184,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5">
+      <c r="A185" t="s">
+        <v>667</v>
+      </c>
+      <c r="B185" t="s">
+        <v>668</v>
+      </c>
+      <c r="C185" t="b">
+        <v>1</v>
+      </c>
+      <c r="D185" t="b" cm="1">
+        <f t="array" ref="D185">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,OR(_xlpm.k=2,_xlpm.k=5,_xlpm.k=8)),"47",AND(_xlpm.r=4,_xlpm.k=7),"478",_xlpm.r=4,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairRowStep(_xlpm.c),SUM(--(_xlpm.s=""))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E185" t="str">
+        <f>IF(D185=C185,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate Sudoku prototype Naked Pair Column to structured step
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{872FFCB4-8498-1641-A2F4-481DDC0891D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172AE5DB-6C70-3845-95A3-DB89180FA18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -84,7 +84,7 @@
     <definedName name="SDKP_ApplyStep">_xlfn.LAMBDA(_xlpm.c,_xlpm.s,_xlfn.LET(_xlpm.removeText,INDEX(_xlpm.s,1,3)&amp;"",_xlpm.targets,INDEX(_xlpm.s,1,4)&amp;"",_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.LET(_xlpm.cur,INDEX(_xlpm.c,_xlpm.r,_xlpm.k)&amp;"",_xlpm.coord,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k,IF(OR(_xlpm.cur="",ISERROR(SEARCH(_xlpm.coord,_xlpm.targets))),_xlpm.cur,_xlfn.LET(_xlpm.chars,MID(_xlpm.cur,_xlfn.SEQUENCE(LEN(_xlpm.cur)),1),_xlfn.TEXTJOIN("",TRUE,_xlfn._xlws.FILTER(_xlpm.chars,ISERROR(SEARCH(_xlpm.chars,_xlpm.removeText)),"")))))))))</definedName>
     <definedName name="SDKP_BasicHint">_xlfn.LAMBDA(_xlpm.c,_xlfn.LET(_xlpm.a,SDKP_Naked(_xlpm.c),_xlpm.b,SDKP_HiddenRow(_xlpm.c),_xlpm.d,SDKP_HiddenCol(_xlpm.c),_xlpm.e,SDKP_HiddenBox(_xlpm.c),IF(_xlpm.a&lt;&gt;"",_xlpm.a,IF(_xlpm.b&lt;&gt;"",_xlpm.b,IF(_xlpm.d&lt;&gt;"",_xlpm.d,_xlpm.e)))))</definedName>
     <definedName name="SDKP_Chain">_xlfn.LAMBDA(_xlpm.board,_xlpm.lim,SDKP_ChainLoop(_xlpm.board,SDK_CandidateMatrix(_xlpm.board),0,_xlpm.lim,""))</definedName>
-    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.claimRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingRowStep(_xlpm.c)),_xlpm.claimRowText,INDEX(_xlpm.claimRowStep,1,5),_xlpm.claimColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingColStep(_xlpm.c)),_xlpm.claimColText,INDEX(_xlpm.claimColStep,1,5),_xlpm.pairRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairRowStep(_xlpm.c)),_xlpm.pairRowText,INDEX(_xlpm.pairRowStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,IF(_xlpm.colText&lt;&gt;"",_xlpm.colStep,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowStep,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColStep,_xlpm.pairRowStep)))),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,IF(_xlpm.colText&lt;&gt;"",_xlpm.colText,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowText,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColText,_xlpm.pairRowText)))),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
+    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.claimRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingRowStep(_xlpm.c)),_xlpm.claimRowText,INDEX(_xlpm.claimRowStep,1,5),_xlpm.claimColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingColStep(_xlpm.c)),_xlpm.claimColText,INDEX(_xlpm.claimColStep,1,5),_xlpm.pairRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairRowStep(_xlpm.c)),_xlpm.pairRowText,INDEX(_xlpm.pairRowStep,1,5),_xlpm.pairColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;"",_xlpm.pairRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairColStep(_xlpm.c)),_xlpm.pairColText,INDEX(_xlpm.pairColStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,IF(_xlpm.colText&lt;&gt;"",_xlpm.colStep,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowStep,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColStep,IF(_xlpm.pairRowText&lt;&gt;"",_xlpm.pairRowStep,_xlpm.pairColStep))))),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,IF(_xlpm.colText&lt;&gt;"",_xlpm.colText,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowText,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColText,IF(_xlpm.pairRowText&lt;&gt;"",_xlpm.pairRowText,_xlpm.pairColText))))),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
     <definedName name="SDKP_ClaimingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_ClaimingColStep(_xlpm.inputCandidates),1,5))</definedName>
     <definedName name="SDKP_ClaimingColStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.i,_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,0,_xlpm.k),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.rs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.rs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*(_xlpm.band-1),_xlpm.bc,1+3*QUOTIENT(_xlpm.k-1,3),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.cc&lt;&gt;_xlpm.k)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.rs&amp;"C"&amp;_xlpm.k),_xlpm.b,3*(_xlpm.band-1)+1+QUOTIENT(_xlpm.k-1,3),_xlpm.displayText,"Claiming column · Column "&amp;_xlpm.k&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".",IF(_xlpm.txt&lt;&gt;"",_xlfn.HSTACK("Claiming column",_xlpm.sourceText,_xlpm.d&amp;"",_xlpm.txt,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_ClaimingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_ClaimingRowStep(_xlpm.inputCandidates),1,5))</definedName>
@@ -97,7 +97,8 @@
     <definedName name="SDKP_HiddenRow">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.k,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))),"Hidden single in row · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in row "&amp;_xlpm.r&amp;"."))))</definedName>
     <definedName name="SDKP_Naked">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.m,LEN(_xlpm.c)=1,_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlfn.TOCOL(_xlpm.m)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.k,MOD(_xlpm.p-1,9)+1,_xlpm.d,INDEX(_xlpm.c,_xlpm.r,_xlpm.k),"Naked single · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · This is the only legal candidate remaining in the square."))))</definedName>
     <definedName name="SDKP_NakedPairBox">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.foundHint,_xlpm.scanIndex,IF(_xlpm.foundHint&lt;&gt;"",_xlpm.foundHint,_xlfn.LET(_xlpm.rowNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.colNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.boxStartRow,1+3*QUOTIENT(_xlpm.rowNum-1,3),_xlpm.boxStartCol,1+3*QUOTIENT(_xlpm.colNum-1,3),_xlpm.unitVals,_xlfn.TOCOL(INDEX(_xlpm.candMatrix,_xlfn.SEQUENCE(3,,_xlpm.boxStartRow),_xlfn.SEQUENCE(,3,_xlpm.boxStartCol)))&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.rowCoords,_xlpm.boxStartRow+QUOTIENT(_xlfn.SEQUENCE(9)-1,3),_xlpm.colCoords,_xlpm.boxStartCol+MOD(_xlfn.SEQUENCE(9)-1,3),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstIndex)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondIndex),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowCoords&amp;"C"&amp;_xlpm.colCoords,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.firstRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.firstIndex-1,3),_xlpm.firstCol,_xlpm.boxStartCol+MOD(_xlpm.firstIndex-1,3),_xlpm.secondRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.secondIndex-1,3),_xlpm.secondCol,_xlpm.boxStartCol+MOD(_xlpm.secondIndex-1,3),_xlpm.boxNum,1+3*QUOTIENT(_xlpm.rowNum-1,3)+QUOTIENT(_xlpm.colNum-1,3),IF(_xlpm.targetText&lt;&gt;"","Naked pair in box · R"&amp;_xlpm.firstRow&amp;"C"&amp;_xlpm.firstCol&amp;" and R"&amp;_xlpm.secondRow&amp;"C"&amp;_xlpm.secondCol&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" in box "&amp;_xlpm.boxNum&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".","")))))))</definedName>
-    <definedName name="SDKP_NakedPairCol">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.foundHint,_xlpm.scanIndex,IF(_xlpm.foundHint&lt;&gt;"",_xlpm.foundHint,_xlfn.LET(_xlpm.colNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.rowNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.unitVals,INDEX(_xlpm.candMatrix,0,_xlpm.colNum)&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstPos)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondPos),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlfn.SEQUENCE(9)&amp;"C"&amp;_xlpm.colNum,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),IF(_xlpm.targetText&lt;&gt;"","Naked pair in column · R"&amp;_xlpm.firstPos&amp;"C"&amp;_xlpm.colNum&amp;" and R"&amp;_xlpm.secondPos&amp;"C"&amp;_xlpm.colNum&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".","")))))))</definedName>
+    <definedName name="SDKP_NakedPairCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_NakedPairColStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_NakedPairColStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.colNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.rowNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.unitVals,INDEX(_xlpm.candMatrix,0,_xlpm.colNum)&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstPos)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondPos),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlfn.SEQUENCE(9)&amp;"C"&amp;_xlpm.colNum,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.sourceText,"R"&amp;_xlpm.firstPos&amp;"C"&amp;_xlpm.colNum&amp;", R"&amp;_xlpm.secondPos&amp;"C"&amp;_xlpm.colNum,_xlpm.displayText,"Naked pair in column · R"&amp;_xlpm.firstPos&amp;"C"&amp;_xlpm.colNum&amp;" and R"&amp;_xlpm.secondPos&amp;"C"&amp;_xlpm.colNum&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".",IF(_xlpm.targetText&lt;&gt;"",_xlfn.HSTACK("Naked pair in column",_xlpm.sourceText,_xlpm.pairText,_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_NakedPairRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_NakedPairRowStep(_xlpm.inputCandidates),1,5))</definedName>
     <definedName name="SDKP_NakedPairRowStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.rowNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.colNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.unitVals,INDEX(_xlpm.candMatrix,_xlpm.rowNum,0)&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(,9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1,1),0),_xlpm.secondPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1,COLUMNS(_xlpm.pairPositions)),0),_xlpm.otherMask,(_xlfn.SEQUENCE(,9)&lt;&gt;_xlpm.firstPos)*(_xlfn.SEQUENCE(,9)&lt;&gt;_xlpm.secondPos),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(,9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlfn.SEQUENCE(,9),_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.sourceText,"R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.firstPos&amp;", R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.secondPos,_xlpm.displayText,"Naked pair in row · R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.firstPos&amp;" and R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.secondPos&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".",IF(_xlpm.targetText&lt;&gt;"",_xlfn.HSTACK("Naked pair in row",_xlpm.sourceText,_xlpm.pairText,_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_PointingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_PointingColStep(_xlpm.inputCandidates),1,5))</definedName>
@@ -185,7 +186,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="669">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="674">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2227,6 +2228,21 @@
   </si>
   <si>
     <t>Exactly two matching cells are required</t>
+  </si>
+  <si>
+    <t>Naked-pair-column step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Structured naked-pair-column apply ignores wording</t>
+  </si>
+  <si>
+    <t>Pair digits and target remove 4/7 from R7C6</t>
+  </si>
+  <si>
+    <t>Naked-pair-column public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Three matching column pairs do not form a naked pair</t>
   </si>
 </sst>
 </file>
@@ -5871,7 +5887,7 @@
       <c r="C45" s="81"/>
       <c r="D45" s="77" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>114 checks passing · 18 on demand</v>
+        <v>118 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="78"/>
       <c r="F45" s="78"/>
@@ -37878,7 +37894,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P185"/>
+  <dimension ref="A1:P189"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -41271,6 +41287,86 @@
       </c>
       <c r="E185" t="str">
         <f>IF(D185=C185,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5">
+      <c r="A186" t="s">
+        <v>669</v>
+      </c>
+      <c r="B186" t="s">
+        <v>662</v>
+      </c>
+      <c r="C186" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D186" t="b" cm="1">
+        <f t="array" ref="D186">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=6,OR(_xlpm.r=2,_xlpm.r=5)),"47",AND(_xlpm.r=7,_xlpm.k=6),"478",_xlpm.k=6,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairColStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Naked pair in column",INDEX(_xlpm.s,1,2)="R2C6, R5C6",INDEX(_xlpm.s,1,3)="47",INDEX(_xlpm.s,1,4)="R7C6",INDEX(_xlpm.s,1,5)="Naked pair in column · R2C6 and R5C6 contain only 4/7 · Remove 4 and 7 from R7C6."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E186" t="str">
+        <f>IF(D186=C186,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5">
+      <c r="A187" t="s">
+        <v>670</v>
+      </c>
+      <c r="B187" t="s">
+        <v>671</v>
+      </c>
+      <c r="C187" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D187" t="b" cm="1">
+        <f t="array" ref="D187">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=6,OR(_xlpm.r=2,_xlpm.r=5)),"47",AND(_xlpm.r=7,_xlpm.k=6),"478",_xlpm.k=6,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairColStep(_xlpm.c),_xlpm.t,_xlfn.HSTACK(INDEX(_xlpm.s,1,1),INDEX(_xlpm.s,1,2),INDEX(_xlpm.s,1,3),INDEX(_xlpm.s,1,4),"wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.c,_xlpm.t),AND(INDEX(_xlpm.after,7,6)="8",INDEX(_xlpm.after,2,6)="47")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E187" t="str">
+        <f>IF(D187=C187,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5">
+      <c r="A188" t="s">
+        <v>672</v>
+      </c>
+      <c r="B188" t="s">
+        <v>666</v>
+      </c>
+      <c r="C188" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D188" t="b" cm="1">
+        <f t="array" ref="D188">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=6,OR(_xlpm.r=2,_xlpm.r=5)),"47",AND(_xlpm.r=7,_xlpm.k=6),"478",_xlpm.k=6,"1235689",TRUE,"123456789"))),SDKP_NakedPairCol(_xlpm.c)=INDEX(SDKP_NakedPairColStep(_xlpm.c),1,5)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E188" t="str">
+        <f>IF(D188=C188,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5">
+      <c r="A189" t="s">
+        <v>673</v>
+      </c>
+      <c r="B189" t="s">
+        <v>668</v>
+      </c>
+      <c r="C189" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D189" t="b" cm="1">
+        <f t="array" ref="D189">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=6,OR(_xlpm.r=2,_xlpm.r=5,_xlpm.r=8)),"47",AND(_xlpm.r=7,_xlpm.k=6),"478",_xlpm.k=6,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairColStep(_xlpm.c),SUM(--(_xlpm.s=""))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E189" t="str">
+        <f>IF(D189=C189,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate Sudoku prototype Naked Pair Box to structured step
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172AE5DB-6C70-3845-95A3-DB89180FA18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D8F55D-81B7-8E49-B10E-C640C2A8F56F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -84,7 +84,7 @@
     <definedName name="SDKP_ApplyStep">_xlfn.LAMBDA(_xlpm.c,_xlpm.s,_xlfn.LET(_xlpm.removeText,INDEX(_xlpm.s,1,3)&amp;"",_xlpm.targets,INDEX(_xlpm.s,1,4)&amp;"",_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.LET(_xlpm.cur,INDEX(_xlpm.c,_xlpm.r,_xlpm.k)&amp;"",_xlpm.coord,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k,IF(OR(_xlpm.cur="",ISERROR(SEARCH(_xlpm.coord,_xlpm.targets))),_xlpm.cur,_xlfn.LET(_xlpm.chars,MID(_xlpm.cur,_xlfn.SEQUENCE(LEN(_xlpm.cur)),1),_xlfn.TEXTJOIN("",TRUE,_xlfn._xlws.FILTER(_xlpm.chars,ISERROR(SEARCH(_xlpm.chars,_xlpm.removeText)),"")))))))))</definedName>
     <definedName name="SDKP_BasicHint">_xlfn.LAMBDA(_xlpm.c,_xlfn.LET(_xlpm.a,SDKP_Naked(_xlpm.c),_xlpm.b,SDKP_HiddenRow(_xlpm.c),_xlpm.d,SDKP_HiddenCol(_xlpm.c),_xlpm.e,SDKP_HiddenBox(_xlpm.c),IF(_xlpm.a&lt;&gt;"",_xlpm.a,IF(_xlpm.b&lt;&gt;"",_xlpm.b,IF(_xlpm.d&lt;&gt;"",_xlpm.d,_xlpm.e)))))</definedName>
     <definedName name="SDKP_Chain">_xlfn.LAMBDA(_xlpm.board,_xlpm.lim,SDKP_ChainLoop(_xlpm.board,SDK_CandidateMatrix(_xlpm.board),0,_xlpm.lim,""))</definedName>
-    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.claimRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingRowStep(_xlpm.c)),_xlpm.claimRowText,INDEX(_xlpm.claimRowStep,1,5),_xlpm.claimColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingColStep(_xlpm.c)),_xlpm.claimColText,INDEX(_xlpm.claimColStep,1,5),_xlpm.pairRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairRowStep(_xlpm.c)),_xlpm.pairRowText,INDEX(_xlpm.pairRowStep,1,5),_xlpm.pairColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;"",_xlpm.pairRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairColStep(_xlpm.c)),_xlpm.pairColText,INDEX(_xlpm.pairColStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,IF(_xlpm.colText&lt;&gt;"",_xlpm.colStep,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowStep,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColStep,IF(_xlpm.pairRowText&lt;&gt;"",_xlpm.pairRowStep,_xlpm.pairColStep))))),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,IF(_xlpm.colText&lt;&gt;"",_xlpm.colText,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowText,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColText,IF(_xlpm.pairRowText&lt;&gt;"",_xlpm.pairRowText,_xlpm.pairColText))))),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",IF(_xlpm.stepText&lt;&gt;"",_xlpm.stepText,SDKP_AdvancedHint(_xlpm.c))),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,IF(_xlpm.stepText&lt;&gt;"",SDKP_ApplyStep(_xlpm.c,_xlpm.step),SDKP_Apply(_xlpm.c,_xlpm.adv)),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
+    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.claimRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingRowStep(_xlpm.c)),_xlpm.claimRowText,INDEX(_xlpm.claimRowStep,1,5),_xlpm.claimColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingColStep(_xlpm.c)),_xlpm.claimColText,INDEX(_xlpm.claimColStep,1,5),_xlpm.pairRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairRowStep(_xlpm.c)),_xlpm.pairRowText,INDEX(_xlpm.pairRowStep,1,5),_xlpm.pairColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;"",_xlpm.pairRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairColStep(_xlpm.c)),_xlpm.pairColText,INDEX(_xlpm.pairColStep,1,5),_xlpm.pairBoxStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;"",_xlpm.pairRowText&lt;&gt;"",_xlpm.pairColText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairBoxStep(_xlpm.c)),_xlpm.pairBoxText,INDEX(_xlpm.pairBoxStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,IF(_xlpm.colText&lt;&gt;"",_xlpm.colStep,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowStep,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColStep,IF(_xlpm.pairRowText&lt;&gt;"",_xlpm.pairRowStep,IF(_xlpm.pairColText&lt;&gt;"",_xlpm.pairColStep,_xlpm.pairBoxStep)))))),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,IF(_xlpm.colText&lt;&gt;"",_xlpm.colText,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowText,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColText,IF(_xlpm.pairRowText&lt;&gt;"",_xlpm.pairRowText,IF(_xlpm.pairColText&lt;&gt;"",_xlpm.pairColText,_xlpm.pairBoxText)))))),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",_xlpm.stepText),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,SDKP_ApplyStep(_xlpm.c,_xlpm.step),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
     <definedName name="SDKP_ClaimingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_ClaimingColStep(_xlpm.inputCandidates),1,5))</definedName>
     <definedName name="SDKP_ClaimingColStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.i,_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,0,_xlpm.k),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.rs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.rs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*(_xlpm.band-1),_xlpm.bc,1+3*QUOTIENT(_xlpm.k-1,3),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.cc&lt;&gt;_xlpm.k)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.rs&amp;"C"&amp;_xlpm.k),_xlpm.b,3*(_xlpm.band-1)+1+QUOTIENT(_xlpm.k-1,3),_xlpm.displayText,"Claiming column · Column "&amp;_xlpm.k&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".",IF(_xlpm.txt&lt;&gt;"",_xlfn.HSTACK("Claiming column",_xlpm.sourceText,_xlpm.d&amp;"",_xlpm.txt,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_ClaimingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_ClaimingRowStep(_xlpm.inputCandidates),1,5))</definedName>
@@ -96,7 +96,8 @@
     <definedName name="SDKP_HiddenCol">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;""))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.r,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;""))),"Hidden single in column · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in column "&amp;_xlpm.k&amp;"."))))</definedName>
     <definedName name="SDKP_HiddenRow">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.k,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))),"Hidden single in row · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in row "&amp;_xlpm.r&amp;"."))))</definedName>
     <definedName name="SDKP_Naked">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.m,LEN(_xlpm.c)=1,_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlfn.TOCOL(_xlpm.m)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.k,MOD(_xlpm.p-1,9)+1,_xlpm.d,INDEX(_xlpm.c,_xlpm.r,_xlpm.k),"Naked single · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · This is the only legal candidate remaining in the square."))))</definedName>
-    <definedName name="SDKP_NakedPairBox">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlfn.REDUCE("",_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.foundHint,_xlpm.scanIndex,IF(_xlpm.foundHint&lt;&gt;"",_xlpm.foundHint,_xlfn.LET(_xlpm.rowNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.colNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.boxStartRow,1+3*QUOTIENT(_xlpm.rowNum-1,3),_xlpm.boxStartCol,1+3*QUOTIENT(_xlpm.colNum-1,3),_xlpm.unitVals,_xlfn.TOCOL(INDEX(_xlpm.candMatrix,_xlfn.SEQUENCE(3,,_xlpm.boxStartRow),_xlfn.SEQUENCE(,3,_xlpm.boxStartCol)))&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.rowCoords,_xlpm.boxStartRow+QUOTIENT(_xlfn.SEQUENCE(9)-1,3),_xlpm.colCoords,_xlpm.boxStartCol+MOD(_xlfn.SEQUENCE(9)-1,3),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstIndex)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondIndex),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowCoords&amp;"C"&amp;_xlpm.colCoords,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.firstRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.firstIndex-1,3),_xlpm.firstCol,_xlpm.boxStartCol+MOD(_xlpm.firstIndex-1,3),_xlpm.secondRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.secondIndex-1,3),_xlpm.secondCol,_xlpm.boxStartCol+MOD(_xlpm.secondIndex-1,3),_xlpm.boxNum,1+3*QUOTIENT(_xlpm.rowNum-1,3)+QUOTIENT(_xlpm.colNum-1,3),IF(_xlpm.targetText&lt;&gt;"","Naked pair in box · R"&amp;_xlpm.firstRow&amp;"C"&amp;_xlpm.firstCol&amp;" and R"&amp;_xlpm.secondRow&amp;"C"&amp;_xlpm.secondCol&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" in box "&amp;_xlpm.boxNum&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".","")))))))</definedName>
+    <definedName name="SDKP_NakedPairBox">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_NakedPairBoxStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_NakedPairBoxStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.rowNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.colNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.boxStartRow,1+3*QUOTIENT(_xlpm.rowNum-1,3),_xlpm.boxStartCol,1+3*QUOTIENT(_xlpm.colNum-1,3),_xlpm.unitVals,_xlfn.TOCOL(INDEX(_xlpm.candMatrix,_xlfn.SEQUENCE(3,,_xlpm.boxStartRow),_xlfn.SEQUENCE(,3,_xlpm.boxStartCol)))&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.rowCoords,_xlpm.boxStartRow+QUOTIENT(_xlfn.SEQUENCE(9)-1,3),_xlpm.colCoords,_xlpm.boxStartCol+MOD(_xlfn.SEQUENCE(9)-1,3),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstIndex)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondIndex),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowCoords&amp;"C"&amp;_xlpm.colCoords,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.firstRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.firstIndex-1,3),_xlpm.firstCol,_xlpm.boxStartCol+MOD(_xlpm.firstIndex-1,3),_xlpm.secondRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.secondIndex-1,3),_xlpm.secondCol,_xlpm.boxStartCol+MOD(_xlpm.secondIndex-1,3),_xlpm.boxNum,1+3*QUOTIENT(_xlpm.rowNum-1,3)+QUOTIENT(_xlpm.colNum-1,3),_xlpm.sourceText,"R"&amp;_xlpm.firstRow&amp;"C"&amp;_xlpm.firstCol&amp;", R"&amp;_xlpm.secondRow&amp;"C"&amp;_xlpm.secondCol,_xlpm.displayText,"Naked pair in box · R"&amp;_xlpm.firstRow&amp;"C"&amp;_xlpm.firstCol&amp;" and R"&amp;_xlpm.secondRow&amp;"C"&amp;_xlpm.secondCol&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" in box "&amp;_xlpm.boxNum&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".",IF(_xlpm.targetText&lt;&gt;"",_xlfn.HSTACK("Naked pair in box",_xlpm.sourceText,_xlpm.pairText,_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_NakedPairCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_NakedPairColStep(_xlpm.inputCandidates),1,5))</definedName>
     <definedName name="SDKP_NakedPairColStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.colNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.rowNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.unitVals,INDEX(_xlpm.candMatrix,0,_xlpm.colNum)&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstPos)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondPos),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlfn.SEQUENCE(9)&amp;"C"&amp;_xlpm.colNum,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.sourceText,"R"&amp;_xlpm.firstPos&amp;"C"&amp;_xlpm.colNum&amp;", R"&amp;_xlpm.secondPos&amp;"C"&amp;_xlpm.colNum,_xlpm.displayText,"Naked pair in column · R"&amp;_xlpm.firstPos&amp;"C"&amp;_xlpm.colNum&amp;" and R"&amp;_xlpm.secondPos&amp;"C"&amp;_xlpm.colNum&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".",IF(_xlpm.targetText&lt;&gt;"",_xlfn.HSTACK("Naked pair in column",_xlpm.sourceText,_xlpm.pairText,_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
     <definedName name="SDKP_NakedPairRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_NakedPairRowStep(_xlpm.inputCandidates),1,5))</definedName>
@@ -186,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="688">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2243,6 +2244,48 @@
   </si>
   <si>
     <t>Three matching column pairs do not form a naked pair</t>
+  </si>
+  <si>
+    <t>Existing naked-pair-box wording maps off-diagonal cells</t>
+  </si>
+  <si>
+    <t>Pair sources and target are mapped in row order</t>
+  </si>
+  <si>
+    <t>Naked-pair-box step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Off-diagonal source pair and target stay separate</t>
+  </si>
+  <si>
+    <t>Structured naked-pair-box apply ignores wording</t>
+  </si>
+  <si>
+    <t>Pair digits remove 4/7 from R3C1</t>
+  </si>
+  <si>
+    <t>Naked-pair-box public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Legacy entry returns the structured display field</t>
+  </si>
+  <si>
+    <t>Three matching box pairs do not form a naked pair</t>
+  </si>
+  <si>
+    <t>Exactly two matching box cells are required</t>
+  </si>
+  <si>
+    <t>Naked-pair-box step preserves middle-box identity</t>
+  </si>
+  <si>
+    <t>Box 5 maps off-diagonal pair to R6C4</t>
+  </si>
+  <si>
+    <t>Chain uses box elimination before the next assignment</t>
+  </si>
+  <si>
+    <t>Box pair removes 4/7 then reveals R3C1=8</t>
   </si>
 </sst>
 </file>
@@ -5887,7 +5930,7 @@
       <c r="C45" s="81"/>
       <c r="D45" s="77" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>118 checks passing · 18 on demand</v>
+        <v>125 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="78"/>
       <c r="F45" s="78"/>
@@ -37894,7 +37937,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P189"/>
+  <dimension ref="A1:P196"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -41367,6 +41410,146 @@
       </c>
       <c r="E189" t="str">
         <f>IF(D189=C189,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5">
+      <c r="A190" t="s">
+        <v>674</v>
+      </c>
+      <c r="B190" t="s">
+        <v>675</v>
+      </c>
+      <c r="C190" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D190" t="b" cm="1">
+        <f t="array" ref="D190">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),SDKP_NakedPairBox(_xlpm.c)="Naked pair in box · R1C2 and R2C3 contain only 4/7 in box 1 · Remove 4 and 7 from R3C1."),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E190" t="str">
+        <f>IF(D190=C190,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5">
+      <c r="A191" t="s">
+        <v>676</v>
+      </c>
+      <c r="B191" t="s">
+        <v>677</v>
+      </c>
+      <c r="C191" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D191" t="b" cm="1">
+        <f t="array" ref="D191">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairBoxStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Naked pair in box",INDEX(_xlpm.s,1,2)="R1C2, R2C3",INDEX(_xlpm.s,1,3)="47",INDEX(_xlpm.s,1,4)="R3C1",INDEX(_xlpm.s,1,5)="Naked pair in box · R1C2 and R2C3 contain only 4/7 in box 1 · Remove 4 and 7 from R3C1."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E191" t="str">
+        <f>IF(D191=C191,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5">
+      <c r="A192" t="s">
+        <v>678</v>
+      </c>
+      <c r="B192" t="s">
+        <v>679</v>
+      </c>
+      <c r="C192" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D192" t="b" cm="1">
+        <f t="array" ref="D192">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairBoxStep(_xlpm.c),_xlpm.action,_xlfn.HSTACK(INDEX(_xlpm.s,1,1),INDEX(_xlpm.s,1,2),INDEX(_xlpm.s,1,3),INDEX(_xlpm.s,1,4),"wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.c,_xlpm.action),AND(INDEX(_xlpm.after,3,1)="8",INDEX(_xlpm.after,1,2)="47",INDEX(_xlpm.after,2,3)="47")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E192" t="str">
+        <f>IF(D192=C192,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5">
+      <c r="A193" t="s">
+        <v>680</v>
+      </c>
+      <c r="B193" t="s">
+        <v>681</v>
+      </c>
+      <c r="C193" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D193" t="b" cm="1">
+        <f t="array" ref="D193">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),SDKP_NakedPairBox(_xlpm.c)=INDEX(SDKP_NakedPairBoxStep(_xlpm.c),1,5)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E193" t="str">
+        <f>IF(D193=C193,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5">
+      <c r="A194" t="s">
+        <v>682</v>
+      </c>
+      <c r="B194" t="s">
+        <v>683</v>
+      </c>
+      <c r="C194" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D194" t="b" cm="1">
+        <f t="array" ref="D194">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairBoxStep(_xlpm.c),SUM(--(_xlpm.s=""))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E194" t="str">
+        <f>IF(D194=C194,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5">
+      <c r="A195" t="s">
+        <v>684</v>
+      </c>
+      <c r="B195" t="s">
+        <v>685</v>
+      </c>
+      <c r="C195" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D195" t="b" cm="1">
+        <f t="array" ref="D195">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,_xlpm.k=5),"47",AND(_xlpm.r=5,_xlpm.k=6),"47",AND(_xlpm.r=6,_xlpm.k=4),"478",AND(_xlpm.r&gt;=4,_xlpm.r&lt;=6,_xlpm.k&gt;=4,_xlpm.k&lt;=6),"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairBoxStep(_xlpm.c),AND(INDEX(_xlpm.s,1,2)="R4C5, R5C6",INDEX(_xlpm.s,1,4)="R6C4",ISNUMBER(SEARCH("in box 5",INDEX(_xlpm.s,1,5))))),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E195" t="str">
+        <f>IF(D195=C195,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5">
+      <c r="A196" t="s">
+        <v>686</v>
+      </c>
+      <c r="B196" t="s">
+        <v>687</v>
+      </c>
+      <c r="C196" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D196" t="b" cm="1">
+        <f t="array" ref="D196">IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,1,""),AND(INDEX(_xlpm.result,10,1)="ASSIGNMENT",INDEX(_xlpm.result,3,1)="8",ISNUMBER(SEARCH("Naked pair in box",INDEX(_xlpm.result,10,5))))),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E196" t="str">
+        <f>IF(D196=C196,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Test Sudoku candidate-chain stop states
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D8F55D-81B7-8E49-B10E-C640C2A8F56F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{734DA805-60B0-1B46-855B-1C6E8F9377BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="688">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="694">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2286,6 +2286,24 @@
   </si>
   <si>
     <t>Box pair removes 4/7 then reveals R3C1=8</t>
+  </si>
+  <si>
+    <t>Chain reports limit with pending elimination</t>
+  </si>
+  <si>
+    <t>Zero budget preserves candidates and pending box hint</t>
+  </si>
+  <si>
+    <t>Chain reports stable without applicable strategy</t>
+  </si>
+  <si>
+    <t>Full candidate matrix has no assignment or elimination</t>
+  </si>
+  <si>
+    <t>Chain reports contradiction for a dead cell</t>
+  </si>
+  <si>
+    <t>Empty R1C1 candidate stops before hint or elimination</t>
   </si>
 </sst>
 </file>
@@ -5930,7 +5948,7 @@
       <c r="C45" s="81"/>
       <c r="D45" s="77" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>125 checks passing · 18 on demand</v>
+        <v>128 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="78"/>
       <c r="F45" s="78"/>
@@ -37937,7 +37955,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P196"/>
+  <dimension ref="A1:P199"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -41550,6 +41568,66 @@
       </c>
       <c r="E196" t="str">
         <f>IF(D196=C196,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5">
+      <c r="A197" t="s">
+        <v>688</v>
+      </c>
+      <c r="B197" t="s">
+        <v>689</v>
+      </c>
+      <c r="C197" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D197" t="b" cm="1">
+        <f t="array" ref="D197">IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,0,""),AND(INDEX(_xlpm.result,10,1)="LIMIT",INDEX(_xlpm.result,10,2)=0,INDEX(_xlpm.result,3,1)="478",ISNUMBER(SEARCH("Naked pair in box",INDEX(_xlpm.result,10,4))),INDEX(_xlpm.result,10,5)="")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E197" t="str">
+        <f>IF(D197=C197,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5">
+      <c r="A198" t="s">
+        <v>690</v>
+      </c>
+      <c r="B198" t="s">
+        <v>691</v>
+      </c>
+      <c r="C198" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D198" t="b">
+        <f>IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"123456789")),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,2,""),AND(INDEX(_xlpm.result,10,1)="STABLE",INDEX(_xlpm.result,10,2)=0,INDEX(_xlpm.result,1,1)="123456789",INDEX(_xlpm.result,10,3)="",INDEX(_xlpm.result,10,4)="",INDEX(_xlpm.result,10,5)="")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E198" t="str">
+        <f>IF(D198=C198,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5">
+      <c r="A199" t="s">
+        <v>692</v>
+      </c>
+      <c r="B199" t="s">
+        <v>693</v>
+      </c>
+      <c r="C199" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D199" t="b" cm="1">
+        <f t="array" ref="D199">IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"","123456789"))),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,2,""),AND(INDEX(_xlpm.result,10,1)="CONTRADICTION",INDEX(_xlpm.result,10,2)=0,INDEX(_xlpm.result,1,1)="",INDEX(_xlpm.result,10,3)="",INDEX(_xlpm.result,10,4)="",INDEX(_xlpm.result,10,5)="")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E199" t="str">
+        <f>IF(D199=C199,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Test Sudoku candidate replay after deletion
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{734DA805-60B0-1B46-855B-1C6E8F9377BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F478D34D-CFB0-EC4A-932F-7F3CC7FFADDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="696">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2304,6 +2304,12 @@
   </si>
   <si>
     <t>Empty R1C1 candidate stops before hint or elimination</t>
+  </si>
+  <si>
+    <t>Chain rebuilds candidates and hint after entry removal</t>
+  </si>
+  <si>
+    <t>R8C3 entry yields STABLE; blank board replays original assignment</t>
   </si>
 </sst>
 </file>
@@ -5948,7 +5954,7 @@
       <c r="C45" s="81"/>
       <c r="D45" s="77" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>128 checks passing · 18 on demand</v>
+        <v>129 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="78"/>
       <c r="F45" s="78"/>
@@ -37955,7 +37961,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P199"/>
+  <dimension ref="A1:P200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -41628,6 +41634,26 @@
       </c>
       <c r="E199" t="str">
         <f>IF(D199=C199,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5">
+      <c r="A200" t="s">
+        <v>694</v>
+      </c>
+      <c r="B200" t="s">
+        <v>695</v>
+      </c>
+      <c r="C200" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D200" t="b">
+        <f>IFERROR(_xlfn.LET(_xlpm.board,'_Engine Master'!$B$27:$J$35,_xlpm.entered,SDK_SetCell(_xlpm.board,8,3,1),_xlpm.afterEntry,SDKP_Chain(_xlpm.entered,8),_xlpm.afterDelete,SDKP_Chain(_xlpm.board,8),AND(INDEX(_xlpm.afterEntry,10,1)="STABLE",INDEX(_xlpm.afterEntry,8,3)="",INDEX(_xlpm.afterEntry,10,3)="",INDEX(_xlpm.afterDelete,10,1)="ASSIGNMENT",INDEX(_xlpm.afterDelete,10,2)=0,INDEX(_xlpm.afterDelete,8,3)="1268",INDEX(_xlpm.afterDelete,10,3)="Hidden single in column · R8C3 = 1 · Digit 1 appears in only one candidate set in column 3.")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E200" t="str">
+        <f>IF(D200=C200,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Test Sudoku conflict recovery after deletion
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F478D34D-CFB0-EC4A-932F-7F3CC7FFADDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4640E7A5-AE28-FA4E-BBC0-CA34C9097FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="698">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2310,6 +2310,12 @@
   </si>
   <si>
     <t>R8C3 entry yields STABLE; blank board replays original assignment</t>
+  </si>
+  <si>
+    <t>Wrong entry stops guidance and removal restores the chain</t>
+  </si>
+  <si>
+    <t>Duplicate 1 flags both cells; clean board returns the original assignment</t>
   </si>
 </sst>
 </file>
@@ -5954,7 +5960,7 @@
       <c r="C45" s="81"/>
       <c r="D45" s="77" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>129 checks passing · 18 on demand</v>
+        <v>130 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="78"/>
       <c r="F45" s="78"/>
@@ -37961,7 +37967,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P200"/>
+  <dimension ref="A1:P201"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -41654,6 +41660,26 @@
       </c>
       <c r="E200" t="str">
         <f>IF(D200=C200,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5">
+      <c r="A201" t="s">
+        <v>696</v>
+      </c>
+      <c r="B201" t="s">
+        <v>697</v>
+      </c>
+      <c r="C201" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D201" t="b" cm="1">
+        <f t="array" ref="D201">IFERROR(_xlfn.LET(_xlpm.board,'_Engine Master'!$B$27:$J$35,_xlpm.wrong,SDK_SetCell(_xlpm.board,2,1,1),_xlpm.wrongChain,SDKP_Chain(_xlpm.wrong,8),_xlpm.recovered,SDKP_Chain(_xlpm.board,8),_xlpm.wrongConflicts,SUM(--_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,SDK_Conflict(_xlpm.wrong,_xlpm.r,_xlpm.k)))),_xlpm.cleanConflicts,SUM(--_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,SDK_Conflict(_xlpm.board,_xlpm.r,_xlpm.k)))),AND(_xlpm.wrongConflicts=2,SDK_Conflict(_xlpm.wrong,1,1),SDK_Conflict(_xlpm.wrong,2,1),INDEX(_xlpm.wrongChain,10,1)="CONTRADICTION",INDEX(_xlpm.wrongChain,10,2)=0,_xlpm.cleanConflicts=0,INDEX(_xlpm.recovered,10,1)="ASSIGNMENT",INDEX(_xlpm.recovered,2,1)="457",INDEX(_xlpm.recovered,10,3)="Hidden single in column · R8C3 = 1 · Digit 1 appears in only one candidate set in column 3.")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E201" t="str">
+        <f>IF(D201=C201,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Test Sudoku chain maximum depth
</commit_message>
<xml_diff>
--- a/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
+++ b/Sudoku/dev-notes/candidate-chain-prototype/sudoku-candidate-chain-structured-slice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/dev-notes/candidate-chain-prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4640E7A5-AE28-FA4E-BBC0-CA34C9097FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACCB7A6A-3B87-D04E-944D-851B5AF3685A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
+    <workbookView xWindow="3280" yWindow="500" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="8" r:id="rId1"/>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="698">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="700">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2316,6 +2316,12 @@
   </si>
   <si>
     <t>Duplicate 1 flags both cells; clean board returns the original assignment</t>
+  </si>
+  <si>
+    <t>Chain enforces the eight-step boundary</t>
+  </si>
+  <si>
+    <t>Nine pointing patterns execute eight steps then retain the ninth as pending</t>
   </si>
 </sst>
 </file>
@@ -5960,7 +5966,7 @@
       <c r="C45" s="81"/>
       <c r="D45" s="77" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>130 checks passing · 18 on demand</v>
+        <v>131 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="78"/>
       <c r="F45" s="78"/>
@@ -37967,7 +37973,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P201"/>
+  <dimension ref="A1:P202"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -41680,6 +41686,26 @@
       </c>
       <c r="E201" t="str">
         <f>IF(D201=C201,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5">
+      <c r="A202" t="s">
+        <v>698</v>
+      </c>
+      <c r="B202" t="s">
+        <v>699</v>
+      </c>
+      <c r="C202" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D202" t="b" cm="1">
+        <f t="array" ref="D202">IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.digits,_xlfn.SEQUENCE(9),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.LET(_xlpm.b,1+3*QUOTIENT(_xlpm.r-1,3),_xlfn.TEXTJOIN("",TRUE,_xlfn._xlws.FILTER(_xlpm.digits,NOT((_xlpm.k&lt;=3)*(_xlpm.digits&gt;=_xlpm.b)*(_xlpm.digits&lt;=_xlpm.b+2)*(_xlpm.digits&lt;&gt;_xlpm.r))))))),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,8,""),_xlpm.log,INDEX(_xlpm.result,10,5),AND(INDEX(_xlpm.result,10,1)="LIMIT",INDEX(_xlpm.result,10,2)=8,INDEX(_xlpm.result,1,4)="23456789",INDEX(_xlpm.result,8,4)="12345679",INDEX(_xlpm.result,9,4)="123456789",ISNUMBER(SEARCH("Pointing row",INDEX(_xlpm.result,10,4))),LEN(_xlpm.log)-LEN(SUBSTITUTE(_xlpm.log,CHAR(10),""))+1=8)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E202" t="str">
+        <f>IF(D202=C202,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>